<commit_message>
Fixed allot of PCB mistakes and added more silkscreen
</commit_message>
<xml_diff>
--- a/BOMs/BOM_ORDER.xlsx
+++ b/BOMs/BOM_ORDER.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Simon\Documents\KiCad\desings\4_DMX node\BOMs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Simon\Documents\KiCad\desings\DMXion 4port node\BOMs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1372D22A-C904-4495-93E3-8CAF3AB35CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD6DB3CE-F99C-4213-9FE7-B49A87125824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{9B84EF14-36DD-40E4-AAD2-543AD15C4A8A}"/>
   </bookViews>
@@ -11408,6 +11408,10 @@
       <c r="R111" s="19">
         <v>14.11</v>
       </c>
+      <c r="S111" s="28">
+        <f>R111+7.9</f>
+        <v>22.009999999999998</v>
+      </c>
     </row>
     <row r="112" spans="1:29" ht="15" customHeight="1">
       <c r="N112" s="14" t="s">

</xml_diff>